<commit_message>
Update emissions factors for SOx and PMS for diesel, biodiesel and methanol ships
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-final-energy.xlsx
+++ b/premise/data/additional_inventories/lci-final-energy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/romain/Github/premise/premise/data/additional_inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{894C046D-FCF4-3340-8C72-6433DB7B3A07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1D64ECF-BCFA-A942-9CD4-F36B938C0129}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2620" yWindow="760" windowWidth="25800" windowHeight="18880" xr2:uid="{B8299F2D-33B8-E148-B485-6429887DEB23}"/>
   </bookViews>
@@ -1258,11 +1258,11 @@
     <t>SOx emissions have been updated to reflect the use of VLSFO.</t>
   </si>
   <si>
-    <t>Wartsila reports an emission factor of about 0.7g NOx/MJ methanol: https://www.wartsila.com/insights/article/next-port-of-call-the-methanol-bunkering-station
-In teh same report, they also report a reduction of 90% of PM emissions compared to using HFO.</t>
+    <t>We assume the absence of sulfur in synthetic diesel. Additionally, according to Petzold et al., 2011, dx.doi.org/10.1021/es2021439, there's a reduction of about 60% in PM emissions relative to using HFO.</t>
   </si>
   <si>
-    <t>We assume the absence of sulfur in synthetic diesel. Additionally, according to Petzold et al., 2011, dx.doi.org/10.1021/es2021439, there's a reduction of about 60% in PM emissions relative to using HFO.</t>
+    <t>Wartsila reports an emission factor of about 0.7g NOx/MJ methanol: https://www.wartsila.com/insights/article/next-port-of-call-the-methanol-bunkering-station
+In the same report, they also report a reduction of 90% of PM emissions compared to using HFO.</t>
   </si>
 </sst>
 </file>
@@ -42546,7 +42546,7 @@
         <v>151</v>
       </c>
       <c r="B2133" s="2" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C2133" s="2"/>
       <c r="D2133" s="2"/>
@@ -43005,8 +43005,8 @@
         <v>71</v>
       </c>
       <c r="B2157" s="3">
-        <f>0.00695*B2138*(1-0.6)</f>
-        <v>7.1282051282051278E-5</v>
+        <f>0.00695*B2138*(1-0.8)</f>
+        <v>3.5641025641025632E-5</v>
       </c>
       <c r="D2157" t="s">
         <v>100</v>
@@ -43024,8 +43024,8 @@
         <v>107</v>
       </c>
       <c r="B2158" s="3">
-        <f>0.0006*B2138*(1-0.6)</f>
-        <v>6.153846153846154E-6</v>
+        <f>0.0006*B2138*(1-0.8)</f>
+        <v>3.0769230769230762E-6</v>
       </c>
       <c r="D2158" t="s">
         <v>100</v>
@@ -43230,7 +43230,7 @@
         <v>151</v>
       </c>
       <c r="B2171" s="38" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C2171" s="2"/>
       <c r="D2171" s="2"/>

</xml_diff>